<commit_message>
slides for lectures 5 and 6 added
</commit_message>
<xml_diff>
--- a/syllabus/ECEN45632_F26_CourseMaterialsInventory.xlsx
+++ b/syllabus/ECEN45632_F26_CourseMaterialsInventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\viby\ecen45632_f26\syllabus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B9EC81-1677-49ED-B26E-39C6641CBACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E91374A-11E7-415D-9A3D-ED076B3ECB97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{BF6D2AD3-84C2-4863-A168-54A8E33BD710}"/>
   </bookViews>
@@ -119,37 +119,37 @@
     <t>Quiz</t>
   </si>
   <si>
-    <t>pdf</t>
-  </si>
-  <si>
-    <t>PS 1</t>
-  </si>
-  <si>
     <t>Exit Ticket</t>
   </si>
   <si>
-    <t>py, pdf</t>
-  </si>
-  <si>
     <t>ipynb</t>
   </si>
   <si>
-    <t>pptx, pdf</t>
-  </si>
-  <si>
-    <t>txt, pdf</t>
-  </si>
-  <si>
     <t>PS 2</t>
   </si>
   <si>
     <t>Q 1</t>
   </si>
   <si>
-    <t xml:space="preserve"> pptx, pdf</t>
-  </si>
-  <si>
     <t>py</t>
+  </si>
+  <si>
+    <t>pptx, pdf, hc</t>
+  </si>
+  <si>
+    <t>txt, pdf, hc</t>
+  </si>
+  <si>
+    <t>pdf, hc</t>
+  </si>
+  <si>
+    <t>py, pdf, hc</t>
+  </si>
+  <si>
+    <t>PS 1, sol</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> pptx, pdf, hc</t>
   </si>
 </sst>
 </file>
@@ -566,7 +566,7 @@
         <v>25</v>
       </c>
       <c r="L6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.45">
@@ -583,19 +583,19 @@
         <v>31</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G8" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="H8" t="s">
+        <v>34</v>
+      </c>
+      <c r="J8" t="s">
+        <v>35</v>
+      </c>
+      <c r="K8" t="s">
         <v>29</v>
-      </c>
-      <c r="J8" t="s">
-        <v>27</v>
-      </c>
-      <c r="K8" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.45">
@@ -606,25 +606,25 @@
         <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E10" t="s">
         <v>31</v>
       </c>
       <c r="F10" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G10" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="H10" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="I10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="J10" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.45">
@@ -641,16 +641,16 @@
         <v>31</v>
       </c>
       <c r="F12" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G12" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="H12" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="I12" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.45">
@@ -667,16 +667,16 @@
         <v>31</v>
       </c>
       <c r="F14" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G14" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="H14" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="I14" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.45">
@@ -720,13 +720,13 @@
         <v>32</v>
       </c>
       <c r="F28" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G28" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="H28" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.45">

</xml_diff>